<commit_message>
Enhance person account definition with screen-proportional width and full detail visibility
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/INFO.xlsx
+++ b/INFO.xlsx
@@ -2181,6 +2181,7 @@
           <t>حساب بانک سپه</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="25" t="inlineStr">
@@ -2206,6 +2207,7 @@
           <t>حساب قرض‌الحسنه مهر ایران</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="25" t="inlineStr">
@@ -2231,6 +2233,7 @@
           <t>حساب بانک ملت</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="25" t="inlineStr">
@@ -2256,6 +2259,7 @@
           <t>حساب پست بانک</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="25" t="inlineStr">
@@ -2281,6 +2285,7 @@
           <t>حساب بانک کشاورزی</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="25" t="inlineStr">
@@ -2298,7 +2303,7 @@
       </c>
       <c r="D14" s="35" t="inlineStr">
         <is>
-          <t>خیر</t>
+          <t>بله</t>
         </is>
       </c>
       <c r="E14" s="28" t="inlineStr">
@@ -2306,6 +2311,7 @@
           <t>حساب آزاد</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="25" t="inlineStr">
@@ -2323,7 +2329,7 @@
       </c>
       <c r="D15" s="34" t="inlineStr">
         <is>
-          <t>خیر</t>
+          <t>بله</t>
         </is>
       </c>
       <c r="E15" s="26" t="inlineStr">
@@ -2331,6 +2337,7 @@
           <t>حساب آزاد</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="25" t="inlineStr">
@@ -2348,7 +2355,7 @@
       </c>
       <c r="D16" s="35" t="inlineStr">
         <is>
-          <t>خیر</t>
+          <t>بله</t>
         </is>
       </c>
       <c r="E16" s="28" t="inlineStr">
@@ -2356,6 +2363,7 @@
           <t>صندوق تنخواه کارگاه</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -12988,7 +12996,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13668,29 +13676,6 @@
       <c r="J36" s="31" t="n"/>
       <c r="K36" s="31" t="n"/>
     </row>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
-    <row r="43"/>
-    <row r="44"/>
-    <row r="45"/>
-    <row r="46"/>
-    <row r="47"/>
-    <row r="48"/>
-    <row r="49"/>
-    <row r="50"/>
-    <row r="51"/>
-    <row r="52"/>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:K2"/>

</xml_diff>